<commit_message>
.\scripts\salvar.ps1 -m "feat(gestao_projetos): vincular formulas dinamicas aos dashboards dos slides 2, 3 e 4 no relatorio mensal de recursos"
</commit_message>
<xml_diff>
--- a/gestao_projetos/execucao_financeira/relatorio_mensal_recursos.xlsx
+++ b/gestao_projetos/execucao_financeira/relatorio_mensal_recursos.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\ARGUS\gestao_projetos\execucao_financeira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56829A7D-7DDB-43F8-8DC7-FC24E4C2FC67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927E82F6-C61D-4960-991C-51B7794AEAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="det_execucao_orcamentaria" sheetId="1" r:id="rId1"/>
-    <sheet name="Slide 2 - Saude do Projeto" sheetId="2" r:id="rId2"/>
-    <sheet name="Slide 3 - Desembolso e Contas" sheetId="3" r:id="rId3"/>
-    <sheet name="Slide 4 - Analise e Atencao" sheetId="4" r:id="rId4"/>
+    <sheet name="Slide 2 - Saude do Projeto" sheetId="11" r:id="rId2"/>
+    <sheet name="Slide 3 - Desembolso e Contas" sheetId="12" r:id="rId3"/>
+    <sheet name="Slide 4 - Analise e Atencao" sheetId="13" r:id="rId4"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="96">
   <si>
     <t>Rubrica</t>
   </si>
@@ -84,9 +85,6 @@
     <t>ISS</t>
   </si>
   <si>
-    <t>Outros Correlatos (Computação em Nuvem)</t>
-  </si>
-  <si>
     <t>Despesas de Suporte Operacional</t>
   </si>
   <si>
@@ -114,42 +112,27 @@
     <t>POLO DE INOVACAO MANAUS - CONVENIO N 002/2026 (BIO CAROCO)</t>
   </si>
   <si>
-    <t>Dashboard de Saude do Projeto - Posicao Fechada em Setembro/2026 (Pronto para Copiar e Colar no Slide 2)</t>
-  </si>
-  <si>
     <t>SALDO DISPONIVEL</t>
   </si>
   <si>
-    <t>R$ 137.823,81</t>
-  </si>
-  <si>
     <t>Fechamento em 30/09/2026</t>
   </si>
   <si>
     <t>RECEITAS RECEBIDAS</t>
   </si>
   <si>
-    <t>R$ 280.500,00</t>
-  </si>
-  <si>
     <t>Aportes acumulados em conta</t>
   </si>
   <si>
     <t>TOTAL EXECUTADO</t>
   </si>
   <si>
-    <t>R$ 147.398,33</t>
-  </si>
-  <si>
     <t>Execucao financeira total</t>
   </si>
   <si>
     <t>RENDIMENTO FINANC.</t>
   </si>
   <si>
-    <t>R$ 4.722,14</t>
-  </si>
-  <si>
     <t>Rendimento liquido aplicacao</t>
   </si>
   <si>
@@ -201,15 +184,9 @@
     <t>TOTAL DO PROJETO</t>
   </si>
   <si>
-    <t>* Posicao em 30/09/2026. Aportado: R$ 280.500,00. Rendimentos liq.: R$ 4.722,14. Saldo em caixa: R$ 137.823,81. Tarifas Empresa/EMBRAPII (R$ 224,50) pagas c/ rendimentos.</t>
-  </si>
-  <si>
     <t>CONV. 002/2026 - DESEMBOLSO E EXECUCAO ORCAMENTARIA (SETEMBRO/2026)</t>
   </si>
   <si>
-    <t>Contas Bancarias: 15334-6 (Empresa), 15335-4 (SEBRAE), 15338-9 (EMBRAPII) - Pronto para Copiar e Colar no Slide 3</t>
-  </si>
-  <si>
     <t>PARCELAS RECEBIDAS (ENTRADAS DE RECEITA)</t>
   </si>
   <si>
@@ -234,9 +211,6 @@
     <t>Ordem Banc.</t>
   </si>
   <si>
-    <t>17/06/2026</t>
-  </si>
-  <si>
     <t>01/04 Emp</t>
   </si>
   <si>
@@ -279,9 +253,6 @@
     <t>TOTAL RECEBIDO</t>
   </si>
   <si>
-    <t>Receitas recebidas: R$ 280.500,00 (49,3% do convenio). Aportes pendentes: R$ 288.500,00.</t>
-  </si>
-  <si>
     <t>RESUMO FINANCEIRO CONSOLIDADO</t>
   </si>
   <si>
@@ -312,9 +283,6 @@
     <t>CONV. 002/2026 - ANALISE DE EXECUCAO E PONTOS DE ATENCAO (SETEMBRO/2026)</t>
   </si>
   <si>
-    <t>Percentuais de Execucao por Rubrica e Destaques Gerenciais - Pronto para Copiar e Colar no Slide 4</t>
-  </si>
-  <si>
     <t>% DE EXECUCAO POR RUBRICA ORCAMENTARIA</t>
   </si>
   <si>
@@ -336,12 +304,6 @@
     <t>EXECUCAO ACUMULADA GERAL</t>
   </si>
   <si>
-    <t>25,9%</t>
-  </si>
-  <si>
-    <t>R$ 147.398,33 executados de R$ 568.100,00 do orcamento total</t>
-  </si>
-  <si>
     <t>SALDO FINANCEIRO DISPONIVEL</t>
   </si>
   <si>
@@ -361,6 +323,18 @@
   </si>
   <si>
     <t>- Despesas Operacionais: Auxiliar Administrativo alocado em DSO (R$ 8,4k executados / 11,6%). Tarifas SEBRAE com R$ 858,32 de saldo.</t>
+  </si>
+  <si>
+    <t>Outros Correlatos (Internet)</t>
+  </si>
+  <si>
+    <t>Dashboard de Saude do Projeto - Posicao Fechada em Setembro/2026 (Vinculado Dinamicamente)</t>
+  </si>
+  <si>
+    <t>Contas Bancarias: 15334-6 (Empresa), 15335-4 (SEBRAE), 15338-9 (EMBRAPII) - Vinculado Dinamicamente</t>
+  </si>
+  <si>
+    <t>Percentuais de Execucao por Rubrica e Destaques Gerenciais - Vinculado Dinamicamente</t>
   </si>
 </sst>
 </file>
@@ -596,7 +570,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -631,160 +605,163 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1019,7 +996,7 @@
                   <c:v>ISS</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Outros Correlatos (Computação em Nuvem)</c:v>
+                  <c:v>Outros Correlatos (Internet)</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>Despesas de Suporte Operacional</c:v>
@@ -1197,7 +1174,7 @@
                   <c:v>ISS</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Outros Correlatos (Computação em Nuvem)</c:v>
+                  <c:v>Outros Correlatos (Internet)</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>Despesas de Suporte Operacional</c:v>
@@ -1239,7 +1216,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>25.936363636363637</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -2001,9 +1978,9 @@
       <sheetName val="orcamento_biocaroco"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3">
         <row r="4">
           <cell r="B4">
@@ -2096,14 +2073,14 @@
             <v>0</v>
           </cell>
         </row>
-        <row r="21">
-          <cell r="E21">
+        <row r="20">
+          <cell r="E20">
             <v>0</v>
           </cell>
         </row>
-        <row r="24">
-          <cell r="E24">
-            <v>8400</v>
+        <row r="23">
+          <cell r="E23">
+            <v>0</v>
           </cell>
         </row>
         <row r="27">
@@ -2134,14 +2111,457 @@
             <v>0</v>
           </cell>
         </row>
-        <row r="33">
-          <cell r="E33">
-            <v>142650</v>
-          </cell>
-        </row>
       </sheetData>
       <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="extrato_bancario"/>
+      <sheetName val="dinamic"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="C1" t="str">
+            <v>mês</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="B2">
+            <v>46204</v>
+          </cell>
+          <cell r="J2">
+            <v>27500</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="J3">
+            <v>-1375</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="J4">
+            <v>-2750</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="J5">
+            <v>184.68</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="J6">
+            <v>-1.34</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="J7">
+            <v>-10.92</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="J8">
+            <v>154.41</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="J9">
+            <v>-6.32</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="J10">
+            <v>88.34</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="J11">
+            <v>-12.34</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="J12">
+            <v>-2800</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="J13">
+            <v>-2800</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="J14">
+            <v>-2800</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="J15">
+            <v>-128.58000000000001</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="J16">
+            <v>-128.57</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="J17">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="J18">
+            <v>-1.7</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="J19">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="J20">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="J21">
+            <v>986.69</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="J22">
+            <v>-1.77</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="J23">
+            <v>-21.31</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="J24">
+            <v>795.84</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="J25">
+            <v>-117.23</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="J26">
+            <v>-20.95</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="J27">
+            <v>249.61</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="J28">
+            <v>-200.93</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="B29">
+            <v>46211</v>
+          </cell>
+          <cell r="J29">
+            <v>150000</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="J30">
+            <v>-12000</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="J31">
+            <v>-12000</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="J32">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="J33">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="J34">
+            <v>-7000</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="J35">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="36">
+          <cell r="J36">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="37">
+          <cell r="J37">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="38">
+          <cell r="J38">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="39">
+          <cell r="J39">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="40">
+          <cell r="J40">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="41">
+          <cell r="J41">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="42">
+          <cell r="J42">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="43">
+          <cell r="J43">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="44">
+          <cell r="J44">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="45">
+          <cell r="J45">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="46">
+          <cell r="J46">
+            <v>-12000</v>
+          </cell>
+        </row>
+        <row r="47">
+          <cell r="J47">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="48">
+          <cell r="J48">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="49">
+          <cell r="J49">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="50">
+          <cell r="J50">
+            <v>-7000</v>
+          </cell>
+        </row>
+        <row r="51">
+          <cell r="J51">
+            <v>-7000</v>
+          </cell>
+        </row>
+        <row r="52">
+          <cell r="J52">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="53">
+          <cell r="J53">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="54">
+          <cell r="J54">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="55">
+          <cell r="J55">
+            <v>-5000</v>
+          </cell>
+        </row>
+        <row r="56">
+          <cell r="J56">
+            <v>-3.16</v>
+          </cell>
+        </row>
+        <row r="57">
+          <cell r="J57">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="58">
+          <cell r="J58">
+            <v>-12.64</v>
+          </cell>
+        </row>
+        <row r="59">
+          <cell r="J59">
+            <v>-28.44</v>
+          </cell>
+        </row>
+        <row r="60">
+          <cell r="J60">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="61">
+          <cell r="J61">
+            <v>-3.16</v>
+          </cell>
+        </row>
+        <row r="62">
+          <cell r="J62">
+            <v>-6.32</v>
+          </cell>
+        </row>
+        <row r="63">
+          <cell r="J63">
+            <v>-18.96</v>
+          </cell>
+        </row>
+        <row r="64">
+          <cell r="J64">
+            <v>334.52</v>
+          </cell>
+        </row>
+        <row r="65">
+          <cell r="J65">
+            <v>972.5</v>
+          </cell>
+        </row>
+        <row r="66">
+          <cell r="J66">
+            <v>-0.01</v>
+          </cell>
+        </row>
+        <row r="67">
+          <cell r="J67">
+            <v>-7.0000000000000007E-2</v>
+          </cell>
+        </row>
+        <row r="68">
+          <cell r="J68">
+            <v>859.45</v>
+          </cell>
+        </row>
+        <row r="69">
+          <cell r="J69">
+            <v>-14.42</v>
+          </cell>
+        </row>
+        <row r="70">
+          <cell r="J70">
+            <v>535.78</v>
+          </cell>
+        </row>
+        <row r="71">
+          <cell r="J71">
+            <v>-32.07</v>
+          </cell>
+        </row>
+        <row r="72">
+          <cell r="B72">
+            <v>46190</v>
+          </cell>
+          <cell r="J72">
+            <v>103000</v>
+          </cell>
+        </row>
+        <row r="73">
+          <cell r="J73">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="74">
+          <cell r="J74">
+            <v>-2125</v>
+          </cell>
+        </row>
+        <row r="75">
+          <cell r="J75">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="76">
+          <cell r="J76">
+            <v>-2000</v>
+          </cell>
+        </row>
+        <row r="77">
+          <cell r="J77">
+            <v>-2125</v>
+          </cell>
+        </row>
+        <row r="78">
+          <cell r="J78">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="79">
+          <cell r="J79">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="80">
+          <cell r="J80">
+            <v>-3.16</v>
+          </cell>
+        </row>
+        <row r="81">
+          <cell r="J81">
+            <v>-3.16</v>
+          </cell>
+        </row>
+        <row r="82">
+          <cell r="J82">
+            <v>-34.5</v>
+          </cell>
+        </row>
+        <row r="83">
+          <cell r="J83">
+            <v>-3.16</v>
+          </cell>
+        </row>
+        <row r="84">
+          <cell r="J84">
+            <v>-6.32</v>
+          </cell>
+        </row>
+        <row r="85">
+          <cell r="J85"/>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2454,7 +2874,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -2463,10 +2883,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2593,7 +3013,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="6">
-        <f>'[2]Cronograma Desembolso'!$E$21</f>
+        <f>'[2]Cronograma Desembolso'!$E$20</f>
         <v>0</v>
       </c>
       <c r="E6" s="6">
@@ -2621,12 +3041,12 @@
         <v>1</v>
       </c>
       <c r="D7" s="6">
-        <f>'[2]Cronograma Desembolso'!$E$24</f>
-        <v>8400</v>
+        <f>'[2]Cronograma Desembolso'!$E$23</f>
+        <v>0</v>
       </c>
       <c r="E7" s="6">
         <f>det_execucao_orcamentaria[[#This Row],[Previsto]]-det_execucao_orcamentaria[[#This Row],[Executado]]</f>
-        <v>-8400</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9">
         <f>IF(det_execucao_orcamentaria[[#This Row],[Previsto]]=0,0,det_execucao_orcamentaria[[#This Row],[Executado]]/det_execucao_orcamentaria[[#This Row],[Previsto]])</f>
@@ -2634,7 +3054,7 @@
       </c>
       <c r="G7" s="9">
         <f>det_execucao_orcamentaria[[#This Row],[Executado]]/det_execucao_orcamentaria[[#Totals],[Previsto]]</f>
-        <v>1.4762741652021089E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -2659,7 +3079,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="6">
         <f>[1]orcamento_biocaroco!$B$18</f>
@@ -2669,7 +3089,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="6">
-        <f>'[2]Cronograma Desembolso'!$E$31</f>
+        <f>'[2]Cronograma Desembolso'!$E$30</f>
         <v>0</v>
       </c>
       <c r="E9" s="6">
@@ -2687,7 +3107,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" s="6">
         <f>[1]orcamento_biocaroco!$B$19</f>
@@ -2697,7 +3117,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="6">
-        <f>'[2]Cronograma Desembolso'!$E$32</f>
+        <f>'[2]Cronograma Desembolso'!$E$31</f>
         <v>0</v>
       </c>
       <c r="E10" s="6">
@@ -2724,25 +3144,25 @@
         <v>1</v>
       </c>
       <c r="D11" s="6">
-        <f>'[2]Cronograma Desembolso'!$E$33</f>
-        <v>142650</v>
+        <f>'[2]Cronograma Desembolso'!$E$32</f>
+        <v>0</v>
       </c>
       <c r="E11" s="6">
         <f>det_execucao_orcamentaria[[#This Row],[Previsto]]-det_execucao_orcamentaria[[#This Row],[Executado]]</f>
-        <v>-137150</v>
+        <v>5500</v>
       </c>
       <c r="F11" s="9">
         <f>IF(det_execucao_orcamentaria[[#This Row],[Previsto]]=0,0,det_execucao_orcamentaria[[#This Row],[Executado]]/det_execucao_orcamentaria[[#This Row],[Previsto]])</f>
-        <v>25.936363636363637</v>
+        <v>0</v>
       </c>
       <c r="G11" s="9">
         <f>det_execucao_orcamentaria[[#This Row],[Executado]]/det_execucao_orcamentaria[[#Totals],[Previsto]]</f>
-        <v>0.25070298769771526</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="B12" s="6">
         <f>[1]orcamento_biocaroco!$B$16</f>
@@ -2770,7 +3190,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="6">
         <f>'[2]Cronograma Desembolso'!$D$28</f>
@@ -2798,7 +3218,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="6">
         <f>[1]orcamento_biocaroco!$B$14</f>
@@ -2826,7 +3246,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="8">
         <f>SUBTOTAL(109,det_execucao_orcamentaria[Previsto])</f>
@@ -2835,22 +3255,22 @@
       <c r="C15" s="8"/>
       <c r="D15" s="8">
         <f>SUBTOTAL(109,det_execucao_orcamentaria[Executado])</f>
-        <v>293700</v>
+        <v>142650</v>
       </c>
       <c r="E15" s="8">
         <f>SUBTOTAL(109,det_execucao_orcamentaria[Disponível])</f>
-        <v>275300</v>
+        <v>426350</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="10">
         <f>SUBTOTAL(109,det_execucao_orcamentaria[%execucao_geral])</f>
-        <v>0.5161687170474516</v>
+        <v>0.25070298769771526</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="D2:D4 F2:F3 F7:F14 D5:D12 D13:D14" calculatedColumn="1"/>
+    <ignoredError sqref="F2:F3 F7:F14 D13:D14 D12 D8" calculatedColumn="1"/>
   </ignoredErrors>
   <drawing r:id="rId1"/>
   <tableParts count="1">
@@ -2860,7 +3280,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD8CF5E1-F34F-488D-AF8D-71DA7BBED7B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4B1B3C7-84EA-4EDE-AF1C-60FA0AC0CB35}">
   <dimension ref="B2:K18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2871,292 +3291,325 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="18.75" x14ac:dyDescent="0.35">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="C5" s="51"/>
+      <c r="D5" s="52" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="52"/>
+      <c r="F5" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="53"/>
+      <c r="H5" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="44"/>
+      <c r="J5" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" s="47"/>
+    </row>
+    <row r="6" spans="2:11" ht="24" x14ac:dyDescent="0.25">
+      <c r="B6" s="45">
+        <f>'Slide 3 - Desembolso e Contas'!J8</f>
+        <v>137823.80999999997</v>
+      </c>
+      <c r="C6" s="46"/>
+      <c r="D6" s="45">
+        <f>'Slide 3 - Desembolso e Contas'!E14</f>
+        <v>280500</v>
+      </c>
+      <c r="E6" s="46"/>
+      <c r="F6" s="45">
+        <f>'Slide 2 - Saude do Projeto'!F17</f>
+        <v>147173.82999999999</v>
+      </c>
+      <c r="G6" s="46"/>
+      <c r="H6" s="45">
+        <f>'Slide 3 - Desembolso e Contas'!J14</f>
+        <v>4722.1400000000003</v>
+      </c>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="46"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="18" t="s">
+      <c r="C7" s="43"/>
+      <c r="D7" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="18"/>
-      <c r="F5" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="19"/>
-      <c r="H5" s="20" t="s">
+      <c r="G7" s="43"/>
+      <c r="H7" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="43"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="I5" s="20"/>
-      <c r="J5" s="21" t="s">
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="39"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="39"/>
+      <c r="J9" s="39"/>
+      <c r="K9" s="39"/>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="40" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="40"/>
+      <c r="D10" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="K5" s="21"/>
-    </row>
-    <row r="6" spans="2:11" ht="24" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16" t="s">
+      <c r="G10" s="41"/>
+      <c r="H10" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="K6" s="16"/>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17" t="s">
+      <c r="I10" s="41"/>
+      <c r="J10" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="K7" s="17"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B9" s="22" t="s">
+      <c r="K10" s="42"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="23"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="24" t="s">
+      <c r="C11" s="28"/>
+      <c r="D11" s="29">
+        <f>det_execucao_orcamentaria!B4</f>
+        <v>458000</v>
+      </c>
+      <c r="E11" s="30"/>
+      <c r="F11" s="29">
+        <f>det_execucao_orcamentaria!D4</f>
+        <v>134250</v>
+      </c>
+      <c r="G11" s="30"/>
+      <c r="H11" s="29">
+        <f>D11-F11</f>
+        <v>323750</v>
+      </c>
+      <c r="I11" s="30"/>
+      <c r="J11" s="31">
+        <f>IF(D11=0,0,F11/D11)</f>
+        <v>0.29312227074235808</v>
+      </c>
+      <c r="K11" s="32"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="25" t="s">
+      <c r="C12" s="33"/>
+      <c r="D12" s="34">
+        <f>det_execucao_orcamentaria!B5</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="35"/>
+      <c r="F12" s="34">
+        <f>det_execucao_orcamentaria!D5</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="35"/>
+      <c r="H12" s="34">
+        <f>D12-F12</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="35"/>
+      <c r="J12" s="36">
+        <f>IF(D12=0,0,F12/D12)</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="37"/>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25" t="s">
+      <c r="C13" s="28"/>
+      <c r="D13" s="29">
+        <f>det_execucao_orcamentaria!B6+det_execucao_orcamentaria!B12</f>
+        <v>9837</v>
+      </c>
+      <c r="E13" s="30"/>
+      <c r="F13" s="29">
+        <f>-([3]extrato_bancario!$J$15 + [3]extrato_bancario!$J$16)</f>
+        <v>257.14999999999998</v>
+      </c>
+      <c r="G13" s="30"/>
+      <c r="H13" s="29">
+        <f>D13-F13</f>
+        <v>9579.85</v>
+      </c>
+      <c r="I13" s="30"/>
+      <c r="J13" s="31">
+        <f>IF(D13=0,0,F13/D13)</f>
+        <v>2.6141099928840093E-2</v>
+      </c>
+      <c r="K13" s="32"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25" t="s">
+      <c r="C14" s="33"/>
+      <c r="D14" s="34">
+        <f>det_execucao_orcamentaria!B11</f>
+        <v>5500</v>
+      </c>
+      <c r="E14" s="35"/>
+      <c r="F14" s="34">
+        <f>-([3]extrato_bancario!$J$3 + [3]extrato_bancario!$J$4)</f>
+        <v>4125</v>
+      </c>
+      <c r="G14" s="35"/>
+      <c r="H14" s="34">
+        <f>D14-F14</f>
+        <v>1375</v>
+      </c>
+      <c r="I14" s="35"/>
+      <c r="J14" s="36">
+        <f>IF(D14=0,0,F14/D14)</f>
+        <v>0.75</v>
+      </c>
+      <c r="K14" s="37"/>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B15" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="25"/>
-      <c r="J10" s="26" t="s">
+      <c r="C15" s="28"/>
+      <c r="D15" s="29">
+        <f>det_execucao_orcamentaria!B14</f>
+        <v>1000</v>
+      </c>
+      <c r="E15" s="30"/>
+      <c r="F15" s="29">
+        <f>-SUM([3]extrato_bancario!$J$56:$J$63)</f>
+        <v>141.68</v>
+      </c>
+      <c r="G15" s="30"/>
+      <c r="H15" s="29">
+        <f>D15-F15</f>
+        <v>858.31999999999994</v>
+      </c>
+      <c r="I15" s="30"/>
+      <c r="J15" s="31">
+        <f>IF(D15=0,0,F15/D15)</f>
+        <v>0.14168</v>
+      </c>
+      <c r="K15" s="32"/>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="K10" s="26"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="33" t="s">
+      <c r="C16" s="33"/>
+      <c r="D16" s="34">
+        <f>det_execucao_orcamentaria!B9+det_execucao_orcamentaria!B10+det_execucao_orcamentaria!B13</f>
+        <v>94663</v>
+      </c>
+      <c r="E16" s="35"/>
+      <c r="F16" s="34">
+        <f>det_execucao_orcamentaria!D13</f>
+        <v>8400</v>
+      </c>
+      <c r="G16" s="35"/>
+      <c r="H16" s="34">
+        <f>D16-F16</f>
+        <v>86263</v>
+      </c>
+      <c r="I16" s="35"/>
+      <c r="J16" s="36">
+        <f>IF(D16=0,0,F16/D16)</f>
+        <v>8.8735831317410183E-2</v>
+      </c>
+      <c r="K16" s="37"/>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B17" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="34">
-        <v>458000</v>
-      </c>
-      <c r="E11" s="35"/>
-      <c r="F11" s="34">
-        <v>134250</v>
-      </c>
-      <c r="G11" s="35"/>
-      <c r="H11" s="34">
-        <v>323750</v>
-      </c>
-      <c r="I11" s="35"/>
-      <c r="J11" s="36">
-        <v>0.29299999999999998</v>
-      </c>
-      <c r="K11" s="37"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29">
-        <v>22400</v>
-      </c>
-      <c r="E12" s="30"/>
-      <c r="F12" s="29">
-        <v>0</v>
-      </c>
-      <c r="G12" s="30"/>
-      <c r="H12" s="29">
-        <v>22400</v>
-      </c>
-      <c r="I12" s="30"/>
-      <c r="J12" s="31">
-        <v>0</v>
-      </c>
-      <c r="K12" s="32"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="33" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="34">
-        <v>8937</v>
-      </c>
-      <c r="E13" s="35"/>
-      <c r="F13" s="34">
-        <v>257.14999999999998</v>
-      </c>
-      <c r="G13" s="35"/>
-      <c r="H13" s="34">
-        <v>8679.85</v>
-      </c>
-      <c r="I13" s="35"/>
-      <c r="J13" s="36">
-        <v>2.9000000000000001E-2</v>
-      </c>
-      <c r="K13" s="37"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="29">
-        <v>5500</v>
-      </c>
-      <c r="E14" s="30"/>
-      <c r="F14" s="29">
-        <v>4125</v>
-      </c>
-      <c r="G14" s="30"/>
-      <c r="H14" s="29">
-        <v>1375</v>
-      </c>
-      <c r="I14" s="30"/>
-      <c r="J14" s="31">
-        <v>0.75</v>
-      </c>
-      <c r="K14" s="32"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="C15" s="33"/>
-      <c r="D15" s="34">
-        <v>1000</v>
-      </c>
-      <c r="E15" s="35"/>
-      <c r="F15" s="34">
-        <v>141.68</v>
-      </c>
-      <c r="G15" s="35"/>
-      <c r="H15" s="34">
-        <v>858.32</v>
-      </c>
-      <c r="I15" s="35"/>
-      <c r="J15" s="36">
-        <v>0.14199999999999999</v>
-      </c>
-      <c r="K15" s="37"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="29">
-        <v>72263</v>
-      </c>
-      <c r="E16" s="30"/>
-      <c r="F16" s="29">
-        <v>8400</v>
-      </c>
-      <c r="G16" s="30"/>
-      <c r="H16" s="29">
-        <v>63863</v>
-      </c>
-      <c r="I16" s="30"/>
-      <c r="J16" s="31">
-        <v>0.11600000000000001</v>
-      </c>
-      <c r="K16" s="32"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39">
-        <v>568100</v>
-      </c>
-      <c r="E17" s="40"/>
-      <c r="F17" s="39">
+      <c r="C17" s="21"/>
+      <c r="D17" s="22">
+        <f>SUM(D11:D16)</f>
+        <v>569000</v>
+      </c>
+      <c r="E17" s="23"/>
+      <c r="F17" s="22">
+        <f>SUM(F11:F16)</f>
         <v>147173.82999999999</v>
       </c>
-      <c r="G17" s="40"/>
-      <c r="H17" s="39">
-        <v>420926.17</v>
-      </c>
-      <c r="I17" s="40"/>
-      <c r="J17" s="41">
-        <v>0.25900000000000001</v>
-      </c>
-      <c r="K17" s="42"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="22">
+        <f>SUM(H11:H16)</f>
+        <v>421826.17</v>
+      </c>
+      <c r="I17" s="23"/>
+      <c r="J17" s="24">
+        <f>F17/D17</f>
+        <v>0.25865347978910369</v>
+      </c>
+      <c r="K17" s="25"/>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="43" t="s">
-        <v>51</v>
+      <c r="B18" s="26" t="str">
+        <f>"* Posicao em 30/09/2026. Aportado: R$ " &amp; TEXT('Slide 3 - Desembolso e Contas'!E14, "#.##0,00") &amp; ". Rendimentos liq.: R$ " &amp; TEXT('Slide 3 - Desembolso e Contas'!J14, "#.##0,00") &amp; ". Saldo em caixa: R$ " &amp; TEXT('Slide 3 - Desembolso e Contas'!J8, "#.##0,00") &amp; ". Tarifas Empresa/EMBRAPII pagas c/ rendimentos."</f>
+        <v>* Posicao em 30/09/2026. Aportado: R$ 280.500,00. Rendimentos liq.: R$ 4.722,14. Saldo em caixa: R$ 137.823,81. Tarifas Empresa/EMBRAPII pagas c/ rendimentos.</v>
       </c>
       <c r="C18" s="27"/>
       <c r="D18" s="27"/>
@@ -3235,7 +3688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05B013D-C228-4299-A3C3-51C9B554EA35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07E70EF6-1A9B-4057-8076-605BF2226F3E}">
   <dimension ref="B2:K15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3246,260 +3699,274 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="18.75" x14ac:dyDescent="0.35">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="H5" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="33"/>
+      <c r="J6" s="34">
+        <f>'Slide 3 - Desembolso e Contas'!J12</f>
+        <v>332.27</v>
+      </c>
+      <c r="K6" s="35"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="C7" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="22" t="s">
+      <c r="D7" s="13">
+        <f>[3]extrato_bancario!$B$72</f>
+        <v>46190</v>
+      </c>
+      <c r="E7" s="16">
+        <f>[3]extrato_bancario!$J$72</f>
+        <v>103000</v>
+      </c>
+      <c r="F7" s="16">
+        <f>E7</f>
+        <v>103000</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="33"/>
+      <c r="J7" s="34">
+        <v>61440.33</v>
+      </c>
+      <c r="K7" s="35"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="H5" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="44" t="s">
+      <c r="C8" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="D8" s="12">
+        <f>[3]extrato_bancario!$B$2</f>
+        <v>46204</v>
+      </c>
+      <c r="E8" s="18">
+        <f>[3]extrato_bancario!$J$2</f>
+        <v>27500</v>
+      </c>
+      <c r="F8" s="18">
+        <f>F7+E8</f>
+        <v>130500</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="21"/>
+      <c r="J8" s="22">
+        <f>SUM([3]extrato_bancario!$J$2:$J$85)</f>
+        <v>137823.80999999997</v>
+      </c>
+      <c r="K8" s="23"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="D6" s="44" t="s">
+      <c r="C9" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="E6" s="44" t="s">
+      <c r="D9" s="13">
+        <f>[3]extrato_bancario!$B$29</f>
+        <v>46211</v>
+      </c>
+      <c r="E9" s="16">
+        <f>[3]extrato_bancario!$J$29</f>
+        <v>150000</v>
+      </c>
+      <c r="F9" s="16">
+        <f>F8+E9</f>
+        <v>280500</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B10" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="44" t="s">
+      <c r="C10" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="I6" s="28"/>
-      <c r="J6" s="29">
+      <c r="D10" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" s="18">
+        <v>27500</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="57" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="39"/>
+      <c r="J10" s="39"/>
+      <c r="K10" s="39"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="16">
+        <v>103000</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="I11" s="33"/>
+      <c r="J11" s="34">
+        <v>4414.24</v>
+      </c>
+      <c r="K11" s="35"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="18">
+        <v>27500</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" s="33"/>
+      <c r="J12" s="34">
         <v>332.27</v>
       </c>
-      <c r="K6" s="30"/>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="47" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="47" t="s">
+      <c r="K12" s="35"/>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="16">
+        <v>103000</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="47" t="s">
-        <v>62</v>
-      </c>
-      <c r="E7" s="48">
-        <v>103000</v>
-      </c>
-      <c r="F7" s="48">
-        <v>103000</v>
-      </c>
-      <c r="H7" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="29">
-        <v>61440.33</v>
-      </c>
-      <c r="K7" s="30"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B8" s="45" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="45" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="49">
-        <v>46029</v>
-      </c>
-      <c r="E8" s="46">
-        <v>27500</v>
-      </c>
-      <c r="F8" s="46">
-        <v>130500</v>
-      </c>
-      <c r="H8" s="38" t="s">
-        <v>81</v>
-      </c>
-      <c r="I8" s="38"/>
-      <c r="J8" s="39">
-        <v>137823.81</v>
-      </c>
-      <c r="K8" s="40"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B9" s="47" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="47" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="50">
-        <v>46241</v>
-      </c>
-      <c r="E9" s="48">
-        <v>150000</v>
-      </c>
-      <c r="F9" s="48">
+      <c r="H13" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="I13" s="33"/>
+      <c r="J13" s="34">
+        <v>24.37</v>
+      </c>
+      <c r="K13" s="35"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="22">
+        <f>SUM(E7:E9)</f>
         <v>280500</v>
       </c>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="45" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="45" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="45" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="46">
-        <v>27500</v>
-      </c>
-      <c r="F10" s="45" t="s">
-        <v>70</v>
-      </c>
-      <c r="H10" s="51" t="s">
-        <v>82</v>
-      </c>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="47" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="47" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="E11" s="48">
-        <v>103000</v>
-      </c>
-      <c r="F11" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="H11" s="52" t="s">
-        <v>83</v>
-      </c>
-      <c r="I11" s="52"/>
-      <c r="J11" s="53">
-        <v>4414.24</v>
-      </c>
-      <c r="K11" s="54"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="45" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="45" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="46">
-        <v>27500</v>
-      </c>
-      <c r="F12" s="45" t="s">
-        <v>70</v>
-      </c>
-      <c r="H12" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="29">
-        <v>332.27</v>
-      </c>
-      <c r="K12" s="30"/>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="47" t="s">
-        <v>74</v>
-      </c>
-      <c r="C13" s="47" t="s">
-        <v>68</v>
-      </c>
-      <c r="D13" s="47" t="s">
-        <v>75</v>
-      </c>
-      <c r="E13" s="48">
-        <v>103000</v>
-      </c>
-      <c r="F13" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="H13" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="I13" s="28"/>
-      <c r="J13" s="29">
-        <v>24.37</v>
-      </c>
-      <c r="K13" s="30"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="38" t="s">
+      <c r="F14" s="23"/>
+      <c r="H14" s="54" t="s">
         <v>76</v>
       </c>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39">
-        <v>280500</v>
-      </c>
-      <c r="F14" s="40"/>
-      <c r="H14" s="52" t="s">
-        <v>86</v>
-      </c>
-      <c r="I14" s="52"/>
-      <c r="J14" s="53">
+      <c r="I14" s="54"/>
+      <c r="J14" s="55">
+        <f>J11+J12-J13</f>
         <v>4722.1400000000003</v>
       </c>
-      <c r="K14" s="54"/>
+      <c r="K14" s="56"/>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="43" t="s">
-        <v>77</v>
+      <c r="B15" s="26" t="str">
+        <f>"Receitas recebidas: R$ " &amp; TEXT(E14, "#.##0,00") &amp; " (" &amp; TEXT(E14/'Slide 2 - Saude do Projeto'!D17, "0,0%") &amp; " do convenio). Aportes pendentes: R$ " &amp; TEXT('Slide 2 - Saude do Projeto'!D17-E14, "#.##0,00") &amp; "."</f>
+        <v>Receitas recebidas: R$ 280.500,00 (49,3% do convenio). Aportes pendentes: R$ 288.500,00.</v>
       </c>
       <c r="C15" s="27"/>
       <c r="D15" s="27"/>
@@ -3508,35 +3975,35 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="B15:F15"/>
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="J8:K8"/>
     <mergeCell ref="H10:K10"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="J11:K11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="B3:K3"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B15:F15"/>
     <mergeCell ref="H5:K5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CB1006-54CE-4FBB-BFF9-2593A8629FBF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF7FC97F-27E4-44E4-B530-E8BA880BF340}">
   <dimension ref="B2:K17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3547,197 +4014,206 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="18.75" x14ac:dyDescent="0.35">
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="48" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B3" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="G5" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" s="62"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="62"/>
+    </row>
+    <row r="6" spans="2:11" ht="26.25" x14ac:dyDescent="0.45">
+      <c r="B6" s="40" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="G6" s="63">
+        <f>'Slide 2 - Saude do Projeto'!J17</f>
+        <v>0.25865347978910369</v>
+      </c>
+      <c r="H6" s="62"/>
+      <c r="I6" s="62"/>
+      <c r="J6" s="62"/>
+      <c r="K6" s="62"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="15">
+        <f>'Slide 2 - Saude do Projeto'!J11</f>
+        <v>0.29312227074235808</v>
+      </c>
+      <c r="G7" s="64" t="str">
+        <f>"R$ " &amp; TEXT('Slide 2 - Saude do Projeto'!F17, "#.##0,00") &amp; " executados de R$ " &amp; TEXT('Slide 2 - Saude do Projeto'!D17, "#.##0,00") &amp; " do orcamento total"</f>
+        <v>R$ 147.173,83 executados de R$ 569.000,00 do orcamento total</v>
+      </c>
+      <c r="H7" s="62"/>
+      <c r="I7" s="62"/>
+      <c r="J7" s="62"/>
+      <c r="K7" s="62"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="14">
+        <f>'Slide 2 - Saude do Projeto'!J12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="15">
+        <f>'Slide 2 - Saude do Projeto'!J14</f>
+        <v>0.75</v>
+      </c>
+      <c r="G9" s="65" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="62"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
+    </row>
+    <row r="10" spans="2:11" ht="26.25" x14ac:dyDescent="0.45">
+      <c r="B10" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="14">
+        <f>'Slide 2 - Saude do Projeto'!J15</f>
+        <v>0.14168</v>
+      </c>
+      <c r="G10" s="66">
+        <f>'Slide 2 - Saude do Projeto'!B6</f>
+        <v>137823.80999999997</v>
+      </c>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B11" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="15">
+        <f>'Slide 2 - Saude do Projeto'!J13</f>
+        <v>2.6141099928840093E-2</v>
+      </c>
+      <c r="G11" s="64" t="s">
+        <v>86</v>
+      </c>
+      <c r="H11" s="62"/>
+      <c r="I11" s="62"/>
+      <c r="J11" s="62"/>
+      <c r="K11" s="62"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="14">
+        <f>'Slide 2 - Saude do Projeto'!J16</f>
+        <v>8.8735831317410183E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="G13" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="14" t="s">
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+    </row>
+    <row r="14" spans="2:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G14" s="59" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="22" t="s">
+      <c r="H14" s="60"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="60"/>
+      <c r="K14" s="60"/>
+    </row>
+    <row r="15" spans="2:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G15" s="59" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="G5" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="H5" s="59"/>
-      <c r="I5" s="59"/>
-      <c r="J5" s="59"/>
-      <c r="K5" s="59"/>
-    </row>
-    <row r="6" spans="2:11" ht="26.25" x14ac:dyDescent="0.45">
-      <c r="B6" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="55"/>
-      <c r="D6" s="55"/>
-      <c r="E6" s="44" t="s">
+      <c r="H15" s="60"/>
+      <c r="I15" s="60"/>
+      <c r="J15" s="60"/>
+      <c r="K15" s="60"/>
+    </row>
+    <row r="16" spans="2:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G16" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="60" t="s">
-        <v>96</v>
-      </c>
-      <c r="H6" s="59"/>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
-    </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="33" t="s">
+      <c r="H16" s="60"/>
+      <c r="I16" s="60"/>
+      <c r="J16" s="60"/>
+      <c r="K16" s="60"/>
+    </row>
+    <row r="17" spans="7:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="57">
-        <v>0.29299999999999998</v>
-      </c>
-      <c r="G7" s="61" t="s">
-        <v>97</v>
-      </c>
-      <c r="H7" s="59"/>
-      <c r="I7" s="59"/>
-      <c r="J7" s="59"/>
-      <c r="K7" s="59"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B8" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B9" s="33" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="57">
-        <v>0.75</v>
-      </c>
-      <c r="G9" s="62" t="s">
-        <v>98</v>
-      </c>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-    </row>
-    <row r="10" spans="2:11" ht="26.25" x14ac:dyDescent="0.45">
-      <c r="B10" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="56">
-        <v>0.14199999999999999</v>
-      </c>
-      <c r="G10" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="H10" s="59"/>
-      <c r="I10" s="59"/>
-      <c r="J10" s="59"/>
-      <c r="K10" s="59"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="33" t="s">
-        <v>93</v>
-      </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="57">
-        <v>2.9000000000000001E-2</v>
-      </c>
-      <c r="G11" s="61" t="s">
-        <v>99</v>
-      </c>
-      <c r="H11" s="59"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="56">
-        <v>0.11600000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="G13" s="64" t="s">
-        <v>100</v>
-      </c>
-      <c r="H13" s="23"/>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23"/>
-      <c r="K13" s="23"/>
-    </row>
-    <row r="14" spans="2:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="65" t="s">
-        <v>101</v>
-      </c>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="66"/>
-    </row>
-    <row r="15" spans="2:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G15" s="65" t="s">
-        <v>102</v>
-      </c>
-      <c r="H15" s="66"/>
-      <c r="I15" s="66"/>
-      <c r="J15" s="66"/>
-      <c r="K15" s="66"/>
-    </row>
-    <row r="16" spans="2:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G16" s="65" t="s">
-        <v>103</v>
-      </c>
-      <c r="H16" s="66"/>
-      <c r="I16" s="66"/>
-      <c r="J16" s="66"/>
-      <c r="K16" s="66"/>
-    </row>
-    <row r="17" spans="7:11" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G17" s="65" t="s">
-        <v>104</v>
-      </c>
-      <c r="H17" s="66"/>
-      <c r="I17" s="66"/>
-      <c r="J17" s="66"/>
-      <c r="K17" s="66"/>
+      <c r="H17" s="60"/>
+      <c r="I17" s="60"/>
+      <c r="J17" s="60"/>
+      <c r="K17" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="21">

</xml_diff>

<commit_message>
feat(gestao_projetos): vincular formulas dinamicas aos dashboards dos slides 2, 3 e 4 no relatorio mensal e perenizar regras orcamentarias
</commit_message>
<xml_diff>
--- a/gestao_projetos/execucao_financeira/relatorio_mensal_recursos.xlsx
+++ b/gestao_projetos/execucao_financeira/relatorio_mensal_recursos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\ARGUS\gestao_projetos\execucao_financeira\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ARGUS\gestao_projetos\execucao_financeira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{927E82F6-C61D-4960-991C-51B7794AEAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA96768-4BCE-45C8-B8BA-1D9C98C8A23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="det_execucao_orcamentaria" sheetId="1" r:id="rId1"/>
@@ -3440,12 +3440,12 @@
       </c>
       <c r="G11" s="30"/>
       <c r="H11" s="29">
-        <f>D11-F11</f>
+        <f t="shared" ref="H11:H16" si="0">D11-F11</f>
         <v>323750</v>
       </c>
       <c r="I11" s="30"/>
       <c r="J11" s="31">
-        <f>IF(D11=0,0,F11/D11)</f>
+        <f t="shared" ref="J11:J16" si="1">IF(D11=0,0,F11/D11)</f>
         <v>0.29312227074235808</v>
       </c>
       <c r="K11" s="32"/>
@@ -3466,12 +3466,12 @@
       </c>
       <c r="G12" s="35"/>
       <c r="H12" s="34">
-        <f>D12-F12</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I12" s="35"/>
       <c r="J12" s="36">
-        <f>IF(D12=0,0,F12/D12)</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K12" s="37"/>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="G13" s="30"/>
       <c r="H13" s="29">
-        <f>D13-F13</f>
+        <f t="shared" si="0"/>
         <v>9579.85</v>
       </c>
       <c r="I13" s="30"/>
       <c r="J13" s="31">
-        <f>IF(D13=0,0,F13/D13)</f>
+        <f t="shared" si="1"/>
         <v>2.6141099928840093E-2</v>
       </c>
       <c r="K13" s="32"/>
@@ -3518,12 +3518,12 @@
       </c>
       <c r="G14" s="35"/>
       <c r="H14" s="34">
-        <f>D14-F14</f>
+        <f t="shared" si="0"/>
         <v>1375</v>
       </c>
       <c r="I14" s="35"/>
       <c r="J14" s="36">
-        <f>IF(D14=0,0,F14/D14)</f>
+        <f t="shared" si="1"/>
         <v>0.75</v>
       </c>
       <c r="K14" s="37"/>
@@ -3544,12 +3544,12 @@
       </c>
       <c r="G15" s="30"/>
       <c r="H15" s="29">
-        <f>D15-F15</f>
+        <f t="shared" si="0"/>
         <v>858.31999999999994</v>
       </c>
       <c r="I15" s="30"/>
       <c r="J15" s="31">
-        <f>IF(D15=0,0,F15/D15)</f>
+        <f t="shared" si="1"/>
         <v>0.14168</v>
       </c>
       <c r="K15" s="32"/>
@@ -3570,12 +3570,12 @@
       </c>
       <c r="G16" s="35"/>
       <c r="H16" s="34">
-        <f>D16-F16</f>
+        <f t="shared" si="0"/>
         <v>86263</v>
       </c>
       <c r="I16" s="35"/>
       <c r="J16" s="36">
-        <f>IF(D16=0,0,F16/D16)</f>
+        <f t="shared" si="1"/>
         <v>8.8735831317410183E-2</v>
       </c>
       <c r="K16" s="37"/>
@@ -3623,11 +3623,49 @@
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="B9:K9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:K13"/>
     <mergeCell ref="B18:K18"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="D15:E15"/>
@@ -3639,49 +3677,11 @@
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="H16:I16"/>
     <mergeCell ref="J16:K16"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="B9:K9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:K17"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -3975,28 +3975,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="H5:K5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="J11:K11"/>
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="H14:I14"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B5:F5"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="E14:F14"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="J7:K7"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -4217,11 +4217,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="G13:K13"/>
-    <mergeCell ref="G14:K14"/>
-    <mergeCell ref="G15:K15"/>
-    <mergeCell ref="G16:K16"/>
-    <mergeCell ref="G17:K17"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B11:D11"/>
@@ -4232,12 +4232,12 @@
     <mergeCell ref="G9:K9"/>
     <mergeCell ref="G10:K10"/>
     <mergeCell ref="G11:K11"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
     <mergeCell ref="B8:D8"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="G14:K14"/>
+    <mergeCell ref="G15:K15"/>
+    <mergeCell ref="G16:K16"/>
+    <mergeCell ref="G17:K17"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>